<commit_message>
fixed pengaturan master data akademik
</commit_message>
<xml_diff>
--- a/docs/test-cases/TC_Kamar_List.xlsx
+++ b/docs/test-cases/TC_Kamar_List.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'List Kamar'!$A$2:$J$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'List Kamar'!$A$2:$J$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1110,172 +1110,226 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
+          <t>Cari by Instansi</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Ada kamar di sebuah instansi (mis. SDIT)</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>1) Seed kamar instansi SDIT
+2) Ketik nama instansi di Cari
+3) Amati hasil</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Keyword=SDIT</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Hasil memuat kamar instansi tsb</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>PRD</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>BUG-018: search by Instansi balik empty padahal data ada (dikonfirmasi manual, pola BUG-001 Mapel). Search by Nama normal</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>TC-KMR-LST-012</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Positif</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
           <t>Cari by PIC</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Ada kamar dgn PIC terisi (guru instansi)</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>1) Seed kamar + pilih PIC (guru pertama)
 2) Ketik nama PIC di Cari
 3) Amati hasil</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Keyword=&lt;nama PIC seed&gt;</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Hasil memuat kamar dgn PIC tsb</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>PRD</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>Belum dijalankan</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>Bergantung instansi punya guru; bila SDIT tak punya guru -&gt; tahap PIC di-skip</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>TC-KMR-LST-012</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>BUG-017: search by PIC balik empty padahal data ada (dikonfirmasi manual). Search by Nama normal; hanya by PIC rusak</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>TC-KMR-LST-013</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Edge</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Cari case-insensitive (huruf kecil) menemukan data</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>Ada kamar dgn nama unik</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>1) Seed kamar nama unik (uppercase QA...)
 2) Ketik versi huruf kecil di Cari
 3) Amati hasil</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Nama=QA&lt;ts&gt;&lt;seq&gt;; keyword=qa&lt;ts&gt;&lt;seq&gt;</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Search tidak case-sensitive -&gt; kamar tetap ditemukan</t>
         </is>
       </c>
-      <c r="H14" s="10" t="inlineStr">
+      <c r="H15" s="10" t="inlineStr">
         <is>
           <t>Asumsi</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>Belum dijalankan</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>PRD tak eksplisit soal case-insensitive -&gt; asumsi konvensi modul lain</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>TC-KMR-LST-013</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>TC-KMR-LST-014</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Negatif</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Cari keyword tidak ada -&gt; halaman kosong</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>List Kamar terbuka</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>1) Ketik keyword acak yang pasti tak match
 2) Amati hasil</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Keyword=ZZZQA000NOTEXIST</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Tidak ada baris; tampil halaman kosong (empty state)</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>PRD</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>Belum dijalankan</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>TC-KMR-LST-014</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>TC-KMR-LST-015</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Positif</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Clear search -&gt; list kembali tampil penuh</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Sudah melakukan search</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>1) Seed kamar
 2) Search nama tsb
@@ -1283,84 +1337,84 @@
 4) Amati list</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Nama=QA&lt;ts&gt;&lt;seq&gt;</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Setelah dikosongkan, list kembali menampilkan banyak baris (tidak ter-filter)</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>PRD</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>Belum dijalankan</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>TC-KMR-LST-015</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>TC-KMR-LST-016</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Edge</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Cari pakai teks Lokasi -&gt; TIDAK menemukan (Lokasi bukan kriteria search)</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Ada kamar dgn Lokasi unik</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>1) Seed kamar + Lokasi unik
 2) Ketik teks Lokasi tsb di Cari
 3) Amati hasil</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>Lokasi=LOK&lt;ts&gt;&lt;seq&gt; (unik); Nama=QA&lt;ts&gt;&lt;seq&gt;</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Kamar TIDAK muncul via pencarian Lokasi (PRD: search hanya Instansi/Nama/PIC) -&gt; halaman kosong</t>
         </is>
       </c>
-      <c r="H17" s="10" t="inlineStr">
+      <c r="H18" s="10" t="inlineStr">
         <is>
           <t>Asumsi</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>Belum dijalankan</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>PRD eksplisit sebut 3 kriteria search (tanpa Lokasi). Jika kamar MALAH muncul = behavior beda dari PRD</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J17"/>
+  <autoFilter ref="A2:J18"/>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
@@ -1374,7 +1428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1546,12 +1600,36 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BUG-017</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Search/cari by PIC balik empty state padahal data ada (pola BUG-001 Mapel). Hanya by PIC; search by Nama normal. Lihat TC-012</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BUG-018</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Search/cari by Instansi balik empty state padahal data ada (pola BUG-001 Mapel). Search by Nama normal. Lihat TC-011</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>Catatan</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>Tanpa kategori security/injection (sesuai kesepakatan)</t>
         </is>

</xml_diff>